<commit_message>
Final update to Table S6 extent area
</commit_message>
<xml_diff>
--- a/oct2026-results tables/territories_by_dataset.xlsx
+++ b/oct2026-results tables/territories_by_dataset.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>New Caledonia</t>
+          <t>French Polynesia</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>French Polynesia</t>
+          <t>New Caledonia</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Wallis and Futuna</t>
+          <t>Mayotte</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Clipperton Island</t>
+          <t>Wallis and Futuna</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Juan de Nova Island</t>
+          <t>Clipperton Island</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Mayotte</t>
+          <t>Juan de Nova Island</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Johnston Atoll</t>
+          <t>Puerto Rico</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Johnston Atoll</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>United States Virgin Islands</t>
+          <t>Palmyra Atoll</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Palmyra Atoll</t>
+          <t>United States Virgin Islands</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Table S9 to summaries
</commit_message>
<xml_diff>
--- a/oct2026-results tables/territories_by_dataset.xlsx
+++ b/oct2026-results tables/territories_by_dataset.xlsx
@@ -10,6 +10,7 @@
     <sheet name="aca_wcmc" sheetId="1" r:id="rId1"/>
     <sheet name="wcmc" sheetId="2" r:id="rId2"/>
     <sheet name="aca_coral" sheetId="3" r:id="rId3"/>
+    <sheet name="aca_wcmc_ssp585" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2491,4 +2492,746 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B61"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>eez_country</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>eez_countries_territories</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Cocos Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Christmas Island</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Serranilla Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Serrana Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bajo Nuevo Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Quitasueño Bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>East Timor</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Oecusse</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Galapagos</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Eritrea</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Doumeira Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>French Polynesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>New Caledonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Mayotte</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Wallis and Futuna</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Clipperton Island</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Juan de Nova Island</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Guadeloupe</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Martinique</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Collectivity of Saint Martin</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Réunion</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Saint-Barthélemy</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Europa Island</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Ile Tromelin</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Bassas da India</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Navassa Island</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Andaman and Nicobar</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Kiribati</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Gilbert Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Kiribati</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Line Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Kiribati</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Phoenix Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Madagascar</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Glorioso Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Saba</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Aruba</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Bonaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Sint-Eustatius</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Sint-Maarten</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Cook Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Niue</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Tokelau</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Republic of Mauritius</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Chagos Archipelago</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Sudan</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Halaib Triangle</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Senkaku Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Abu musa, Greater and Lesser Tunb</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Turks and Caicos Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>British Virgin Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Bermuda</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Cayman Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Anguilla</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Pitcairn</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Montserrat</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Hawaii</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>American Samoa</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Guam</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Northern Mariana Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Puerto Rico</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>United States Virgin Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Palmyra Atoll</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Johnston Atoll</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Wake Island / Enenkio</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Howland and Baker Islands</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Jarvis Island</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>